<commit_message>
feat: modernización BH 2026, design system y Operación
Health gate Outlook, plazos por período, locks, MailLedger, sync
Excel↔PG, stages 0/6/8–10 vía services, UI Apple-like y UX Docentes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/BD-DOCENTES.xlsx
+++ b/BD-DOCENTES.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M265"/>
+  <dimension ref="A1:M266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15381,10 +15381,8 @@
           <t>17255004-5</t>
         </is>
       </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>17255004</t>
-        </is>
+      <c r="B265" t="n">
+        <v>17255004</v>
       </c>
       <c r="C265" t="inlineStr">
         <is>
@@ -15426,6 +15424,51 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>16454383-8</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>16454383</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Sanchéz Villar,Roberto Carlos</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>rcsanchezvillar@gmail.com</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>+56948857113</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr"/>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>TALCA</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>mcasanovar@santotomas.cl</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr"/>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="inlineStr"/>
+      <c r="L266" t="inlineStr"/>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>[AUTO] Agregado 2026-06-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: operación mensual con Postgres, catálogo DP y avisos de correo
El mes se opera con preview de provisionados, Avance por tipo y DP
resuelto por sede; el paso 1 avisa antes de enviar si falta correo.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/BD-DOCENTES.xlsx
+++ b/BD-DOCENTES.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M266"/>
+  <dimension ref="A1:M267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15391,7 +15391,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>c.bustosmoreira@gmail.com</t>
+          <t>cbustos27@santotomas.cl</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
@@ -15420,7 +15420,7 @@
       <c r="L265" t="inlineStr"/>
       <c r="M265" t="inlineStr">
         <is>
-          <t>[AUTO] Agregado 2026-05-25</t>
+          <t>[AUTO] Agregado 2026-05-25 | Canal institucional pedido 2026-08-18: cbustos27@santotomas.cl. Gmail de respaldo: c.bustosmoreira@gmail.com.</t>
         </is>
       </c>
     </row>
@@ -15469,6 +15469,51 @@
         </is>
       </c>
     </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>18157697-9</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>18157697</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Argandoña Zumaran,Leonardo Alberto</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>leonardo.argandona@hotmail.com</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>+56990124566</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr"/>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>VALDIVIA</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>saleuy@santotomas.cl</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr"/>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="inlineStr"/>
+      <c r="L267" t="inlineStr"/>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>[AUTO] Agregado 2026-08-21</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>